<commit_message>
Add Pool finals results (26 Oct)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014GvXJk1znZiefEz7vJwK1C
</commit_message>
<xml_diff>
--- a/data/Tomstars_House_Cup_2026_gsheet.xlsx
+++ b/data/Tomstars_House_Cup_2026_gsheet.xlsx
@@ -368,7 +368,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I304"/>
+  <dimension ref="A1:I308"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="36.140625" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -11624,6 +11624,150 @@
       </c>
       <c r="I304" s="4" t="n">
         <v>46322.54170138889</v>
+      </c>
+    </row>
+    <row r="305">
+      <c r="A305" t="inlineStr">
+        <is>
+          <t>e1a06732-276d-4a9a-af5b-9fd7463691ef</t>
+        </is>
+      </c>
+      <c r="B305" t="inlineStr">
+        <is>
+          <t>Blue</t>
+        </is>
+      </c>
+      <c r="C305" t="n">
+        <v>100</v>
+      </c>
+      <c r="D305" t="inlineStr">
+        <is>
+          <t>Pool (Men) - Final Winner</t>
+        </is>
+      </c>
+      <c r="E305" t="inlineStr">
+        <is>
+          <t>Olympia</t>
+        </is>
+      </c>
+      <c r="F305" t="n">
+        <v>1</v>
+      </c>
+      <c r="G305" t="inlineStr">
+        <is>
+          <t>Ankit Tyagi</t>
+        </is>
+      </c>
+      <c r="I305" s="4" t="n">
+        <v>46321.70833333334</v>
+      </c>
+    </row>
+    <row r="306">
+      <c r="A306" t="inlineStr">
+        <is>
+          <t>bd293ca7-4ee0-45ce-8d5e-e62cfc6f2cf7</t>
+        </is>
+      </c>
+      <c r="B306" t="inlineStr">
+        <is>
+          <t>Blue</t>
+        </is>
+      </c>
+      <c r="C306" t="n">
+        <v>50</v>
+      </c>
+      <c r="D306" t="inlineStr">
+        <is>
+          <t>Pool (Men) - Final Runner Up</t>
+        </is>
+      </c>
+      <c r="E306" t="inlineStr">
+        <is>
+          <t>Olympia</t>
+        </is>
+      </c>
+      <c r="F306" t="n">
+        <v>1</v>
+      </c>
+      <c r="G306" t="inlineStr">
+        <is>
+          <t>Hiraman Chorghade</t>
+        </is>
+      </c>
+      <c r="I306" s="4" t="n">
+        <v>46321.70834490741</v>
+      </c>
+    </row>
+    <row r="307">
+      <c r="A307" t="inlineStr">
+        <is>
+          <t>ecfbdb85-9ad0-4a75-83c3-ea738f86e28a</t>
+        </is>
+      </c>
+      <c r="B307" t="inlineStr">
+        <is>
+          <t>Green</t>
+        </is>
+      </c>
+      <c r="C307" t="n">
+        <v>100</v>
+      </c>
+      <c r="D307" t="inlineStr">
+        <is>
+          <t>Pool (Women) - Final Winner</t>
+        </is>
+      </c>
+      <c r="E307" t="inlineStr">
+        <is>
+          <t>Olympia</t>
+        </is>
+      </c>
+      <c r="F307" t="n">
+        <v>1</v>
+      </c>
+      <c r="G307" t="inlineStr">
+        <is>
+          <t>Monika Jambhulkar</t>
+        </is>
+      </c>
+      <c r="I307" s="4" t="n">
+        <v>46321.70835648148</v>
+      </c>
+    </row>
+    <row r="308">
+      <c r="A308" t="inlineStr">
+        <is>
+          <t>f45dda16-f570-486b-8e66-fe9a91fbb4b3</t>
+        </is>
+      </c>
+      <c r="B308" t="inlineStr">
+        <is>
+          <t>Blue</t>
+        </is>
+      </c>
+      <c r="C308" t="n">
+        <v>50</v>
+      </c>
+      <c r="D308" t="inlineStr">
+        <is>
+          <t>Pool (Women) - Final Runner Up</t>
+        </is>
+      </c>
+      <c r="E308" t="inlineStr">
+        <is>
+          <t>Olympia</t>
+        </is>
+      </c>
+      <c r="F308" t="n">
+        <v>1</v>
+      </c>
+      <c r="G308" t="inlineStr">
+        <is>
+          <t>Ankita Agrawal</t>
+        </is>
+      </c>
+      <c r="I308" s="4" t="n">
+        <v>46321.70836805556</v>
       </c>
     </row>
   </sheetData>
@@ -11745,17 +11889,6 @@
           <t>TBA</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr"/>
-      <c r="F2" t="inlineStr"/>
-      <c r="G2" t="inlineStr"/>
-      <c r="H2" t="inlineStr"/>
-      <c r="I2" t="inlineStr"/>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr"/>
-      <c r="L2" t="inlineStr"/>
-      <c r="M2" t="inlineStr"/>
-      <c r="N2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -11773,17 +11906,6 @@
           <t>TBA</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr"/>
-      <c r="E3" t="inlineStr"/>
-      <c r="F3" t="inlineStr"/>
-      <c r="G3" t="inlineStr"/>
-      <c r="H3" t="inlineStr"/>
-      <c r="I3" t="inlineStr"/>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr"/>
-      <c r="L3" t="inlineStr"/>
-      <c r="M3" t="inlineStr"/>
-      <c r="N3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -11806,16 +11928,11 @@
           <t>Today</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr">
         <is>
           <t>Game Room</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr"/>
-      <c r="H4" t="inlineStr"/>
-      <c r="I4" t="inlineStr"/>
-      <c r="J4" t="inlineStr"/>
       <c r="K4" t="inlineStr">
         <is>
           <t>Yogesh Nimbalkar</t>
@@ -11858,7 +11975,6 @@
           <t>Tomorrow</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr">
         <is>
           <t>Game Room</t>
@@ -11884,10 +12000,6 @@
           <t>White</t>
         </is>
       </c>
-      <c r="K5" t="inlineStr"/>
-      <c r="L5" t="inlineStr"/>
-      <c r="M5" t="inlineStr"/>
-      <c r="N5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -11905,17 +12017,6 @@
           <t>TBA</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr"/>
-      <c r="E6" t="inlineStr"/>
-      <c r="F6" t="inlineStr"/>
-      <c r="G6" t="inlineStr"/>
-      <c r="H6" t="inlineStr"/>
-      <c r="I6" t="inlineStr"/>
-      <c r="J6" t="inlineStr"/>
-      <c r="K6" t="inlineStr"/>
-      <c r="L6" t="inlineStr"/>
-      <c r="M6" t="inlineStr"/>
-      <c r="N6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -11933,17 +12034,6 @@
           <t>TBA</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr"/>
-      <c r="E7" t="inlineStr"/>
-      <c r="F7" t="inlineStr"/>
-      <c r="G7" t="inlineStr"/>
-      <c r="H7" t="inlineStr"/>
-      <c r="I7" t="inlineStr"/>
-      <c r="J7" t="inlineStr"/>
-      <c r="K7" t="inlineStr"/>
-      <c r="L7" t="inlineStr"/>
-      <c r="M7" t="inlineStr"/>
-      <c r="N7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -11976,14 +12066,6 @@
           <t>Majauli</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr"/>
-      <c r="H8" t="inlineStr"/>
-      <c r="I8" t="inlineStr"/>
-      <c r="J8" t="inlineStr"/>
-      <c r="K8" t="inlineStr"/>
-      <c r="L8" t="inlineStr"/>
-      <c r="M8" t="inlineStr"/>
-      <c r="N8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -12006,12 +12088,6 @@
           <t>Today</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr"/>
-      <c r="F9" t="inlineStr"/>
-      <c r="G9" t="inlineStr"/>
-      <c r="H9" t="inlineStr"/>
-      <c r="I9" t="inlineStr"/>
-      <c r="J9" t="inlineStr"/>
       <c r="K9" t="inlineStr">
         <is>
           <t>Ankita Agrawal</t>
@@ -12046,20 +12122,34 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>TBA</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr"/>
-      <c r="E10" t="inlineStr"/>
-      <c r="F10" t="inlineStr"/>
-      <c r="G10" t="inlineStr"/>
-      <c r="H10" t="inlineStr"/>
-      <c r="I10" t="inlineStr"/>
-      <c r="J10" t="inlineStr"/>
-      <c r="K10" t="inlineStr"/>
-      <c r="L10" t="inlineStr"/>
-      <c r="M10" t="inlineStr"/>
-      <c r="N10" t="inlineStr"/>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>26 Oct 2026</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>Ankit Tyagi</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>Blue</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>Hiraman Chorghade</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>Blue</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -12074,20 +12164,34 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>TBA</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr"/>
-      <c r="E11" t="inlineStr"/>
-      <c r="F11" t="inlineStr"/>
-      <c r="G11" t="inlineStr"/>
-      <c r="H11" t="inlineStr"/>
-      <c r="I11" t="inlineStr"/>
-      <c r="J11" t="inlineStr"/>
-      <c r="K11" t="inlineStr"/>
-      <c r="L11" t="inlineStr"/>
-      <c r="M11" t="inlineStr"/>
-      <c r="N11" t="inlineStr"/>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>26 Oct 2026</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>Monika Jambhulkar</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>Green</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>Ankita Agrawal</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>Blue</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -12140,10 +12244,6 @@
           <t>Blue</t>
         </is>
       </c>
-      <c r="K12" t="inlineStr"/>
-      <c r="L12" t="inlineStr"/>
-      <c r="M12" t="inlineStr"/>
-      <c r="N12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -12196,10 +12296,6 @@
           <t>Blue</t>
         </is>
       </c>
-      <c r="K13" t="inlineStr"/>
-      <c r="L13" t="inlineStr"/>
-      <c r="M13" t="inlineStr"/>
-      <c r="N13" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add Jenga Women, Table Tennis and Chess finals results; fix Jenga name corrections
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014GvXJk1znZiefEz7vJwK1C
</commit_message>
<xml_diff>
--- a/data/Tomstars_House_Cup_2026_gsheet.xlsx
+++ b/data/Tomstars_House_Cup_2026_gsheet.xlsx
@@ -368,7 +368,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I308"/>
+  <dimension ref="A1:I318"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="36.140625" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -11547,7 +11547,7 @@
       </c>
       <c r="G302" t="inlineStr">
         <is>
-          <t>Nitin Patil</t>
+          <t>Nitin Sapnar</t>
         </is>
       </c>
       <c r="I302" s="4" t="n">
@@ -11768,6 +11768,366 @@
       </c>
       <c r="I308" s="4" t="n">
         <v>46321.70836805556</v>
+      </c>
+    </row>
+    <row r="309">
+      <c r="A309" t="inlineStr">
+        <is>
+          <t>1a379f6b-691f-4f1b-8d5c-661a1eb8509b</t>
+        </is>
+      </c>
+      <c r="B309" t="inlineStr">
+        <is>
+          <t>White</t>
+        </is>
+      </c>
+      <c r="C309" t="n">
+        <v>100</v>
+      </c>
+      <c r="D309" t="inlineStr">
+        <is>
+          <t>Jenga (Women) - Final Winner</t>
+        </is>
+      </c>
+      <c r="E309" t="inlineStr">
+        <is>
+          <t>Olympia</t>
+        </is>
+      </c>
+      <c r="F309" t="n">
+        <v>1</v>
+      </c>
+      <c r="G309" t="inlineStr">
+        <is>
+          <t>Sapana Hushare</t>
+        </is>
+      </c>
+      <c r="I309" s="4" t="n">
+        <v>46323.5</v>
+      </c>
+    </row>
+    <row r="310">
+      <c r="A310" t="inlineStr">
+        <is>
+          <t>2ed41412-9eb2-4314-8e98-d429163eb815</t>
+        </is>
+      </c>
+      <c r="B310" t="inlineStr">
+        <is>
+          <t>White</t>
+        </is>
+      </c>
+      <c r="C310" t="n">
+        <v>50</v>
+      </c>
+      <c r="D310" t="inlineStr">
+        <is>
+          <t>Jenga (Women) - Final Runner Up</t>
+        </is>
+      </c>
+      <c r="E310" t="inlineStr">
+        <is>
+          <t>Olympia</t>
+        </is>
+      </c>
+      <c r="F310" t="n">
+        <v>1</v>
+      </c>
+      <c r="G310" t="inlineStr">
+        <is>
+          <t>Sneha Deshpande</t>
+        </is>
+      </c>
+      <c r="I310" s="4" t="n">
+        <v>46323.50001157408</v>
+      </c>
+    </row>
+    <row r="311">
+      <c r="A311" t="inlineStr">
+        <is>
+          <t>239ce6c2-8595-48bc-8766-acd6fe325039</t>
+        </is>
+      </c>
+      <c r="B311" t="inlineStr">
+        <is>
+          <t>Blue</t>
+        </is>
+      </c>
+      <c r="C311" t="n">
+        <v>100</v>
+      </c>
+      <c r="D311" t="inlineStr">
+        <is>
+          <t>Table Tennis (Women) - Final Winner</t>
+        </is>
+      </c>
+      <c r="E311" t="inlineStr">
+        <is>
+          <t>Olympia</t>
+        </is>
+      </c>
+      <c r="F311" t="n">
+        <v>1</v>
+      </c>
+      <c r="G311" t="inlineStr">
+        <is>
+          <t>Aditi Sabnis</t>
+        </is>
+      </c>
+      <c r="I311" s="4" t="n">
+        <v>46321.75</v>
+      </c>
+    </row>
+    <row r="312">
+      <c r="A312" t="inlineStr">
+        <is>
+          <t>d78f9b7b-0b09-4a4c-ab0f-17abe9c6b7d9</t>
+        </is>
+      </c>
+      <c r="B312" t="inlineStr">
+        <is>
+          <t>Green</t>
+        </is>
+      </c>
+      <c r="C312" t="n">
+        <v>50</v>
+      </c>
+      <c r="D312" t="inlineStr">
+        <is>
+          <t>Table Tennis (Women) - Final Runner Up</t>
+        </is>
+      </c>
+      <c r="E312" t="inlineStr">
+        <is>
+          <t>Olympia</t>
+        </is>
+      </c>
+      <c r="F312" t="n">
+        <v>1</v>
+      </c>
+      <c r="G312" t="inlineStr">
+        <is>
+          <t>Shristi Painaik</t>
+        </is>
+      </c>
+      <c r="I312" s="4" t="n">
+        <v>46321.75001157408</v>
+      </c>
+    </row>
+    <row r="313">
+      <c r="A313" t="inlineStr">
+        <is>
+          <t>ce404da6-66ba-4cae-85df-fc2cbd30ab96</t>
+        </is>
+      </c>
+      <c r="B313" t="inlineStr">
+        <is>
+          <t>Blue</t>
+        </is>
+      </c>
+      <c r="C313" t="n">
+        <v>100</v>
+      </c>
+      <c r="D313" t="inlineStr">
+        <is>
+          <t>Table Tennis (Men) - Final Winner</t>
+        </is>
+      </c>
+      <c r="E313" t="inlineStr">
+        <is>
+          <t>Olympia</t>
+        </is>
+      </c>
+      <c r="F313" t="n">
+        <v>1</v>
+      </c>
+      <c r="G313" t="inlineStr">
+        <is>
+          <t>Ankit Tyagi</t>
+        </is>
+      </c>
+      <c r="I313" s="4" t="n">
+        <v>46321.77083333334</v>
+      </c>
+    </row>
+    <row r="314">
+      <c r="A314" t="inlineStr">
+        <is>
+          <t>05d48971-6e02-4235-9fa1-2ad876aecf0d</t>
+        </is>
+      </c>
+      <c r="B314" t="inlineStr">
+        <is>
+          <t>White</t>
+        </is>
+      </c>
+      <c r="C314" t="n">
+        <v>50</v>
+      </c>
+      <c r="D314" t="inlineStr">
+        <is>
+          <t>Table Tennis (Men) - Final Runner Up</t>
+        </is>
+      </c>
+      <c r="E314" t="inlineStr">
+        <is>
+          <t>Olympia</t>
+        </is>
+      </c>
+      <c r="F314" t="n">
+        <v>1</v>
+      </c>
+      <c r="G314" t="inlineStr">
+        <is>
+          <t>Satyam Kesarwani</t>
+        </is>
+      </c>
+      <c r="I314" s="4" t="n">
+        <v>46321.77084490741</v>
+      </c>
+    </row>
+    <row r="315">
+      <c r="A315" t="inlineStr">
+        <is>
+          <t>2a5ccbb1-1c2d-4d70-8908-fe8f03222c22</t>
+        </is>
+      </c>
+      <c r="B315" t="inlineStr">
+        <is>
+          <t>Blue</t>
+        </is>
+      </c>
+      <c r="C315" t="n">
+        <v>100</v>
+      </c>
+      <c r="D315" t="inlineStr">
+        <is>
+          <t>Chess (Men) - Final Winner</t>
+        </is>
+      </c>
+      <c r="E315" t="inlineStr">
+        <is>
+          <t>Olympia</t>
+        </is>
+      </c>
+      <c r="F315" t="n">
+        <v>1</v>
+      </c>
+      <c r="G315" t="inlineStr">
+        <is>
+          <t>Ankit Tyagi</t>
+        </is>
+      </c>
+      <c r="I315" s="4" t="n">
+        <v>46321.66666666666</v>
+      </c>
+    </row>
+    <row r="316">
+      <c r="A316" t="inlineStr">
+        <is>
+          <t>6275dc52-2691-4496-9940-d7d874807dc1</t>
+        </is>
+      </c>
+      <c r="B316" t="inlineStr">
+        <is>
+          <t>White</t>
+        </is>
+      </c>
+      <c r="C316" t="n">
+        <v>50</v>
+      </c>
+      <c r="D316" t="inlineStr">
+        <is>
+          <t>Chess (Men) - Final Runner Up</t>
+        </is>
+      </c>
+      <c r="E316" t="inlineStr">
+        <is>
+          <t>Olympia</t>
+        </is>
+      </c>
+      <c r="F316" t="n">
+        <v>1</v>
+      </c>
+      <c r="G316" t="inlineStr">
+        <is>
+          <t>Ajay Bharti</t>
+        </is>
+      </c>
+      <c r="I316" s="4" t="n">
+        <v>46321.66667824074</v>
+      </c>
+    </row>
+    <row r="317">
+      <c r="A317" t="inlineStr">
+        <is>
+          <t>c96f37b1-ecb1-43cc-b45a-82bbe35be8fe</t>
+        </is>
+      </c>
+      <c r="B317" t="inlineStr">
+        <is>
+          <t>White</t>
+        </is>
+      </c>
+      <c r="C317" t="n">
+        <v>100</v>
+      </c>
+      <c r="D317" t="inlineStr">
+        <is>
+          <t>Chess (Women) - Final Winner</t>
+        </is>
+      </c>
+      <c r="E317" t="inlineStr">
+        <is>
+          <t>Olympia</t>
+        </is>
+      </c>
+      <c r="F317" t="n">
+        <v>1</v>
+      </c>
+      <c r="G317" t="inlineStr">
+        <is>
+          <t>Ambika Tipare</t>
+        </is>
+      </c>
+      <c r="I317" s="4" t="n">
+        <v>46321.6875</v>
+      </c>
+    </row>
+    <row r="318">
+      <c r="A318" t="inlineStr">
+        <is>
+          <t>ac98f496-df9f-4471-a610-c7ba188c0935</t>
+        </is>
+      </c>
+      <c r="B318" t="inlineStr">
+        <is>
+          <t>Green</t>
+        </is>
+      </c>
+      <c r="C318" t="n">
+        <v>50</v>
+      </c>
+      <c r="D318" t="inlineStr">
+        <is>
+          <t>Chess (Women) - Final Runner Up</t>
+        </is>
+      </c>
+      <c r="E318" t="inlineStr">
+        <is>
+          <t>Olympia</t>
+        </is>
+      </c>
+      <c r="F318" t="n">
+        <v>1</v>
+      </c>
+      <c r="G318" t="inlineStr">
+        <is>
+          <t>Kalyani Tipare</t>
+        </is>
+      </c>
+      <c r="I318" s="4" t="n">
+        <v>46321.68751157408</v>
       </c>
     </row>
   </sheetData>
@@ -11945,7 +12305,7 @@
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>Nitin Patil</t>
+          <t>Nitin Sapnar</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
@@ -11967,14 +12327,15 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Scheduled</t>
+          <t>Completed</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Tomorrow</t>
-        </is>
-      </c>
+          <t>28 Oct 2026</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr">
         <is>
           <t>Game Room</t>
@@ -11996,6 +12357,26 @@
         </is>
       </c>
       <c r="J5" t="inlineStr">
+        <is>
+          <t>White</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>Sapana Hushare</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>White</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>Sneha Deshpande</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
         <is>
           <t>White</t>
         </is>
@@ -12014,7 +12395,34 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>TBA</t>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>26 Oct 2026</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr"/>
+      <c r="F6" t="inlineStr"/>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>Ankit Tyagi</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>Blue</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>Ajay Bharti</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>White</t>
         </is>
       </c>
     </row>
@@ -12031,7 +12439,34 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>TBA</t>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>26 Oct 2026</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr"/>
+      <c r="F7" t="inlineStr"/>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>Ambika Tipare</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>White</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>Kalyani Tipare</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>Green</t>
         </is>
       </c>
     </row>
@@ -12206,19 +12641,15 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Scheduled</t>
+          <t>Completed</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Today</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>3:00 PM</t>
-        </is>
-      </c>
+          <t>26 Oct 2026</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr"/>
       <c r="F12" t="inlineStr">
         <is>
           <t>Game Room</t>
@@ -12242,6 +12673,26 @@
       <c r="J12" t="inlineStr">
         <is>
           <t>Blue</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>Ankit Tyagi</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>Blue</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>Satyam Kesarwani</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>White</t>
         </is>
       </c>
     </row>
@@ -12258,19 +12709,15 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Scheduled</t>
+          <t>Completed</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Today</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>5:00 PM</t>
-        </is>
-      </c>
+          <t>26 Oct 2026</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr"/>
       <c r="F13" t="inlineStr">
         <is>
           <t>Game Room</t>
@@ -12294,6 +12741,26 @@
       <c r="J13" t="inlineStr">
         <is>
           <t>Blue</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>Aditi Sabnis</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>Blue</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>Shristi Painaik</t>
+        </is>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>Green</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Darts and Carrom Men finals results
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014GvXJk1znZiefEz7vJwK1C
</commit_message>
<xml_diff>
--- a/data/Tomstars_House_Cup_2026_gsheet.xlsx
+++ b/data/Tomstars_House_Cup_2026_gsheet.xlsx
@@ -368,7 +368,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I318"/>
+  <dimension ref="A1:I324"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="36.140625" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -12128,6 +12128,222 @@
       </c>
       <c r="I318" s="4" t="n">
         <v>46321.68751157408</v>
+      </c>
+    </row>
+    <row r="319">
+      <c r="A319" t="inlineStr">
+        <is>
+          <t>c448a7c7-7e39-4632-aed4-eab40c1f9fe5</t>
+        </is>
+      </c>
+      <c r="B319" t="inlineStr">
+        <is>
+          <t>Red</t>
+        </is>
+      </c>
+      <c r="C319" t="n">
+        <v>100</v>
+      </c>
+      <c r="D319" t="inlineStr">
+        <is>
+          <t>Darts (Men) - Final Winner</t>
+        </is>
+      </c>
+      <c r="E319" t="inlineStr">
+        <is>
+          <t>Olympia</t>
+        </is>
+      </c>
+      <c r="F319" t="n">
+        <v>1</v>
+      </c>
+      <c r="G319" t="inlineStr">
+        <is>
+          <t>Ritesh Nalawade</t>
+        </is>
+      </c>
+      <c r="I319" s="4" t="n">
+        <v>46321.625</v>
+      </c>
+    </row>
+    <row r="320">
+      <c r="A320" t="inlineStr">
+        <is>
+          <t>4edbcc6b-eaf6-4a12-8472-c0e5474fb2e5</t>
+        </is>
+      </c>
+      <c r="B320" t="inlineStr">
+        <is>
+          <t>Green</t>
+        </is>
+      </c>
+      <c r="C320" t="n">
+        <v>50</v>
+      </c>
+      <c r="D320" t="inlineStr">
+        <is>
+          <t>Darts (Men) - Final Runner Up</t>
+        </is>
+      </c>
+      <c r="E320" t="inlineStr">
+        <is>
+          <t>Olympia</t>
+        </is>
+      </c>
+      <c r="F320" t="n">
+        <v>1</v>
+      </c>
+      <c r="G320" t="inlineStr">
+        <is>
+          <t>Vinod Balesgol</t>
+        </is>
+      </c>
+      <c r="I320" s="4" t="n">
+        <v>46321.62501157408</v>
+      </c>
+    </row>
+    <row r="321">
+      <c r="A321" t="inlineStr">
+        <is>
+          <t>19374d2c-68eb-4a5a-8ba1-1061682d69f5</t>
+        </is>
+      </c>
+      <c r="B321" t="inlineStr">
+        <is>
+          <t>White</t>
+        </is>
+      </c>
+      <c r="C321" t="n">
+        <v>100</v>
+      </c>
+      <c r="D321" t="inlineStr">
+        <is>
+          <t>Darts (Women) - Final Winner</t>
+        </is>
+      </c>
+      <c r="E321" t="inlineStr">
+        <is>
+          <t>Olympia</t>
+        </is>
+      </c>
+      <c r="F321" t="n">
+        <v>1</v>
+      </c>
+      <c r="G321" t="inlineStr">
+        <is>
+          <t>Sneha Deshpande</t>
+        </is>
+      </c>
+      <c r="I321" s="4" t="n">
+        <v>46321.64583333334</v>
+      </c>
+    </row>
+    <row r="322">
+      <c r="A322" t="inlineStr">
+        <is>
+          <t>998fc53f-b746-4686-bb1c-228c45f246d6</t>
+        </is>
+      </c>
+      <c r="B322" t="inlineStr">
+        <is>
+          <t>Green</t>
+        </is>
+      </c>
+      <c r="C322" t="n">
+        <v>50</v>
+      </c>
+      <c r="D322" t="inlineStr">
+        <is>
+          <t>Darts (Women) - Final Runner Up</t>
+        </is>
+      </c>
+      <c r="E322" t="inlineStr">
+        <is>
+          <t>Olympia</t>
+        </is>
+      </c>
+      <c r="F322" t="n">
+        <v>1</v>
+      </c>
+      <c r="G322" t="inlineStr">
+        <is>
+          <t>Preeti Kerkar</t>
+        </is>
+      </c>
+      <c r="I322" s="4" t="n">
+        <v>46321.64584490741</v>
+      </c>
+    </row>
+    <row r="323">
+      <c r="A323" t="inlineStr">
+        <is>
+          <t>4f84bedf-4464-4a2d-800a-ebfc823ef7a4</t>
+        </is>
+      </c>
+      <c r="B323" t="inlineStr">
+        <is>
+          <t>White</t>
+        </is>
+      </c>
+      <c r="C323" t="n">
+        <v>100</v>
+      </c>
+      <c r="D323" t="inlineStr">
+        <is>
+          <t>Carrom (Men) - Final Winner</t>
+        </is>
+      </c>
+      <c r="E323" t="inlineStr">
+        <is>
+          <t>Olympia</t>
+        </is>
+      </c>
+      <c r="F323" t="n">
+        <v>1</v>
+      </c>
+      <c r="G323" t="inlineStr">
+        <is>
+          <t>Ajay Bharti</t>
+        </is>
+      </c>
+      <c r="I323" s="4" t="n">
+        <v>46322.70833333334</v>
+      </c>
+    </row>
+    <row r="324">
+      <c r="A324" t="inlineStr">
+        <is>
+          <t>fde83fe5-fa00-4bd9-8f52-ce8183bb07cf</t>
+        </is>
+      </c>
+      <c r="B324" t="inlineStr">
+        <is>
+          <t>Blue</t>
+        </is>
+      </c>
+      <c r="C324" t="n">
+        <v>50</v>
+      </c>
+      <c r="D324" t="inlineStr">
+        <is>
+          <t>Carrom (Men) - Final Runner Up</t>
+        </is>
+      </c>
+      <c r="E324" t="inlineStr">
+        <is>
+          <t>Olympia</t>
+        </is>
+      </c>
+      <c r="F324" t="n">
+        <v>1</v>
+      </c>
+      <c r="G324" t="inlineStr">
+        <is>
+          <t>Rohit Mane</t>
+        </is>
+      </c>
+      <c r="I324" s="4" t="n">
+        <v>46322.70834490741</v>
       </c>
     </row>
   </sheetData>
@@ -12246,7 +12462,33 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>TBA</t>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>26 Oct 2026</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr"/>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>Ritesh Nalawade</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>Red</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>Vinod Balesgol</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>Green</t>
         </is>
       </c>
     </row>
@@ -12263,7 +12505,33 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>TBA</t>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>26 Oct 2026</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr"/>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>Sneha Deshpande</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>White</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>Preeti Kerkar</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>Green</t>
         </is>
       </c>
     </row>
@@ -12335,7 +12603,6 @@
           <t>28 Oct 2026</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr">
         <is>
           <t>Game Room</t>
@@ -12403,8 +12670,6 @@
           <t>26 Oct 2026</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr"/>
-      <c r="F6" t="inlineStr"/>
       <c r="K6" t="inlineStr">
         <is>
           <t>Ankit Tyagi</t>
@@ -12447,8 +12712,6 @@
           <t>26 Oct 2026</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr"/>
-      <c r="F7" t="inlineStr"/>
       <c r="K7" t="inlineStr">
         <is>
           <t>Ambika Tipare</t>
@@ -12483,22 +12746,38 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Scheduled</t>
+          <t>Completed</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Today</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>4:30 PM</t>
-        </is>
-      </c>
+          <t>27 Oct 2026</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr"/>
       <c r="F8" t="inlineStr">
         <is>
           <t>Majauli</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>Ajay Bharti</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>White</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>Rohit Mane</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>Blue</t>
         </is>
       </c>
     </row>
@@ -12649,7 +12928,6 @@
           <t>26 Oct 2026</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr"/>
       <c r="F12" t="inlineStr">
         <is>
           <t>Game Room</t>
@@ -12717,7 +12995,6 @@
           <t>26 Oct 2026</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr"/>
       <c r="F13" t="inlineStr">
         <is>
           <t>Game Room</t>

</xml_diff>